<commit_message>
Update Trading Journal.xlsx 2026-08-16 20:28:10
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="log" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="stocklist" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="log" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stocklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -583,6 +583,33 @@
         <v>2</v>
       </c>
       <c r="G5" s="1" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>2645</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>長榮航太</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>193.5</v>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>3K反轉</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr"/>
+      <c r="G6" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-16 20:28:37
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -608,7 +608,9 @@
           <t>3K反轉</t>
         </is>
       </c>
-      <c r="F6" s="1" t="inlineStr"/>
+      <c r="F6" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="G6" s="1" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-17 13:37:40
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -428,7 +428,7 @@
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -612,6 +612,39 @@
         <v>1</v>
       </c>
       <c r="G6" s="1" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>8039</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>台虹</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>213</v>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>巧妙點</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="1" t="inlineStr">
+        <is>
+          <t>開盤有巧妙點</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-17 13:43:25
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -645,6 +645,35 @@
           <t>開盤有巧妙點</t>
         </is>
       </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>8039</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>台虹</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>256.5</v>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>停利賣出</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-17 14:36:06
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -674,6 +674,35 @@
         <v>1</v>
       </c>
       <c r="G8" s="1" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>3441</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>聯一光</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>84.90000000000001</v>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>漲幅達標</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-18 09:42:20
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -703,6 +703,35 @@
         <v>3</v>
       </c>
       <c r="G9" s="1" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>6226</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>光鼎</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>20.45</v>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>3K反轉</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="G10" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-18 10:23:19
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -732,6 +732,39 @@
         <v>10</v>
       </c>
       <c r="G10" s="1" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>2645</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>長榮航太</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>178.5</v>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>停損賣出</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="1" t="inlineStr">
+        <is>
+          <t>停損</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-19 21:13:05
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -763,6 +763,39 @@
       <c r="G11" s="1" t="inlineStr">
         <is>
           <t>停損</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>1303</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>南亞</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="n">
+        <v>190</v>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>反向島狀</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="1" t="inlineStr">
+        <is>
+          <t>停利</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-21 17:18:30
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -798,6 +798,64 @@
           <t>停利</t>
         </is>
       </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>3605</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>宏致</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="n">
+        <v>107.5</v>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>巧妙點</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" s="1" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>2484</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>希華</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="n">
+        <v>77.3</v>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>3K反轉</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="G14" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-21 17:20:22
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -856,6 +856,35 @@
         <v>3</v>
       </c>
       <c r="G14" s="1" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>3362</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>先進光</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>180</v>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>3K反轉</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G15" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-24 17:42:40
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -885,6 +885,35 @@
         <v>2</v>
       </c>
       <c r="G15" s="1" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>4566</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>時碩工業</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="n">
+        <v>67</v>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>停損賣出</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="G16" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-24 17:43:22
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -894,24 +894,24 @@
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>4566</t>
+          <t>3441</t>
         </is>
       </c>
       <c r="C16" s="1" t="inlineStr">
         <is>
-          <t>時碩工業</t>
+          <t>聯一光</t>
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>67</v>
+        <v>112</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>停損賣出</t>
+          <t>停利賣出</t>
         </is>
       </c>
       <c r="F16" s="1" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G16" s="1" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-24 17:44:29
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -913,7 +913,11 @@
       <c r="F16" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G16" s="1" t="inlineStr"/>
+      <c r="G16" s="1" t="inlineStr">
+        <is>
+          <t>乖離過大調節</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-24 21:02:31
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -580,7 +580,7 @@
         </is>
       </c>
       <c r="F5" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5" s="1" t="inlineStr"/>
     </row>
@@ -918,6 +918,35 @@
           <t>乖離過大調節</t>
         </is>
       </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>4566</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>時碩工業</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="n">
+        <v>66.8</v>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>停損賣出</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-27 10:45:46
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -423,8 +423,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
@@ -1042,33 +1042,33 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>00408A</t>
+          <t>5483</t>
         </is>
       </c>
       <c r="C21" s="1" t="inlineStr">
         <is>
-          <t>主動第一金優股息</t>
+          <t>中美晶</t>
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>111</v>
+        <v>180</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>三白兵</t>
+          <t>停損賣出</t>
         </is>
       </c>
       <c r="F21" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G21" s="1" t="inlineStr">
         <is>
-          <t>test</t>
+          <t>停損</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-27 12:47:48
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1071,6 +1071,35 @@
           <t>停損</t>
         </is>
       </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t>8261</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>富鼎</t>
+        </is>
+      </c>
+      <c r="D22" s="1" t="n">
+        <v>185.5</v>
+      </c>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>KD高腳</t>
+        </is>
+      </c>
+      <c r="F22" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-27 13:03:35
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1100,6 +1100,35 @@
         <v>1</v>
       </c>
       <c r="G22" s="1" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>3532</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t>台勝科</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="n">
+        <v>392</v>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>KD高腳</t>
+        </is>
+      </c>
+      <c r="F23" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-27 13:19:58
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1129,6 +1129,35 @@
         <v>1</v>
       </c>
       <c r="G23" s="1" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>3605</t>
+        </is>
+      </c>
+      <c r="C24" s="1" t="inlineStr">
+        <is>
+          <t>宏致</t>
+        </is>
+      </c>
+      <c r="D24" s="1" t="n">
+        <v>118.5</v>
+      </c>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>3K反轉</t>
+        </is>
+      </c>
+      <c r="F24" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-27 14:51:48
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -1128,7 +1128,11 @@
       <c r="F23" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G23" s="1" t="inlineStr"/>
+      <c r="G23" s="1" t="inlineStr">
+        <is>
+          <t>迴旋KD</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-28 12:36:49
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1162,6 +1162,33 @@
         <v>1</v>
       </c>
       <c r="G24" s="1" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
+        <is>
+          <t>2484</t>
+        </is>
+      </c>
+      <c r="C25" s="1" t="inlineStr">
+        <is>
+          <t>希華</t>
+        </is>
+      </c>
+      <c r="D25" s="1" t="n">
+        <v>77.90000000000001</v>
+      </c>
+      <c r="E25" s="1" t="inlineStr">
+        <is>
+          <t>停利賣出</t>
+        </is>
+      </c>
+      <c r="F25" s="1" t="inlineStr"/>
+      <c r="G25" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-28 12:37:47
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1187,8 +1187,39 @@
           <t>停利賣出</t>
         </is>
       </c>
-      <c r="F25" s="1" t="inlineStr"/>
+      <c r="F25" s="1" t="n">
+        <v>3</v>
+      </c>
       <c r="G25" s="1" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
+        <is>
+          <t>3441</t>
+        </is>
+      </c>
+      <c r="C26" s="1" t="inlineStr">
+        <is>
+          <t>聯一光</t>
+        </is>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>132.5</v>
+      </c>
+      <c r="E26" s="1" t="inlineStr">
+        <is>
+          <t>陰K加碼</t>
+        </is>
+      </c>
+      <c r="F26" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-28 13:49:49
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1220,6 +1220,35 @@
         <v>1</v>
       </c>
       <c r="G26" s="1" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
+        <is>
+          <t>5351</t>
+        </is>
+      </c>
+      <c r="C27" s="1" t="inlineStr">
+        <is>
+          <t>鈺創</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="n">
+        <v>116</v>
+      </c>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t>巧妙點</t>
+        </is>
+      </c>
+      <c r="F27" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-28 15:29:57
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,16 +419,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -454,15 +455,20 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>買賣方向</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>進出手法</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>買賣張數</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -489,13 +495,18 @@
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
           <t>島狀反轉</t>
         </is>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="G2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G2" s="1" t="inlineStr"/>
+      <c r="H2" s="1" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -518,13 +529,18 @@
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
           <t>停利賣出</t>
         </is>
       </c>
-      <c r="F3" s="1" t="n">
+      <c r="G3" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G3" s="1" t="inlineStr"/>
+      <c r="H3" s="1" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -547,13 +563,18 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
           <t>3K反轉</t>
         </is>
       </c>
-      <c r="F4" s="1" t="n">
+      <c r="G4" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G4" s="1" t="inlineStr"/>
+      <c r="H4" s="1" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -576,13 +597,18 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
           <t>等價進場買入</t>
         </is>
       </c>
-      <c r="F5" s="1" t="n">
+      <c r="G5" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G5" s="1" t="inlineStr"/>
+      <c r="H5" s="1" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -605,13 +631,18 @@
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
           <t>巧妙點</t>
         </is>
       </c>
-      <c r="F6" s="1" t="n">
+      <c r="G6" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G6" s="1" t="inlineStr">
+      <c r="H6" s="1" t="inlineStr">
         <is>
           <t>開盤有巧妙點</t>
         </is>
@@ -638,13 +669,18 @@
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
           <t>漲幅達標</t>
         </is>
       </c>
-      <c r="F7" s="1" t="n">
+      <c r="G7" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="G7" s="1" t="inlineStr"/>
+      <c r="H7" s="1" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -667,13 +703,18 @@
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
           <t>島狀反轉</t>
         </is>
       </c>
-      <c r="F8" s="1" t="n">
+      <c r="G8" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G8" s="1" t="inlineStr"/>
+      <c r="H8" s="1" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -696,13 +737,18 @@
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
           <t>KD高腳</t>
         </is>
       </c>
-      <c r="F9" s="1" t="n">
+      <c r="G9" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="G9" s="1" t="inlineStr"/>
+      <c r="H9" s="1" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -725,13 +771,18 @@
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
           <t>3K反轉</t>
         </is>
       </c>
-      <c r="F10" s="1" t="n">
+      <c r="G10" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="1" t="inlineStr"/>
+      <c r="H10" s="1" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -754,13 +805,18 @@
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
           <t>停利賣出</t>
         </is>
       </c>
-      <c r="F11" s="1" t="n">
+      <c r="G11" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G11" s="1" t="inlineStr"/>
+      <c r="H11" s="1" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -783,13 +839,18 @@
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
           <t>3K反轉</t>
         </is>
       </c>
-      <c r="F12" s="1" t="n">
+      <c r="G12" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="G12" s="1" t="inlineStr"/>
+      <c r="H12" s="1" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -812,13 +873,18 @@
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
           <t>停損賣出</t>
         </is>
       </c>
-      <c r="F13" s="1" t="n">
+      <c r="G13" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G13" s="1" t="inlineStr">
+      <c r="H13" s="1" t="inlineStr">
         <is>
           <t>停損</t>
         </is>
@@ -845,13 +911,18 @@
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
           <t>反向島狀</t>
         </is>
       </c>
-      <c r="F14" s="1" t="n">
+      <c r="G14" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G14" s="1" t="inlineStr">
+      <c r="H14" s="1" t="inlineStr">
         <is>
           <t>停利</t>
         </is>
@@ -878,13 +949,18 @@
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
           <t>巧妙點</t>
         </is>
       </c>
-      <c r="F15" s="1" t="n">
+      <c r="G15" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G15" s="1" t="inlineStr"/>
+      <c r="H15" s="1" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
@@ -907,13 +983,18 @@
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="inlineStr">
+        <is>
           <t>3K反轉</t>
         </is>
       </c>
-      <c r="F16" s="1" t="n">
+      <c r="G16" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="G16" s="1" t="inlineStr"/>
+      <c r="H16" s="1" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
@@ -936,13 +1017,18 @@
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
           <t>停利賣出</t>
         </is>
       </c>
-      <c r="F17" s="1" t="n">
+      <c r="G17" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G17" s="1" t="inlineStr">
+      <c r="H17" s="1" t="inlineStr">
         <is>
           <t>乖離過大調節</t>
         </is>
@@ -969,13 +1055,18 @@
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F18" s="1" t="inlineStr">
+        <is>
           <t>停損賣出</t>
         </is>
       </c>
-      <c r="F18" s="1" t="n">
+      <c r="G18" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="G18" s="1" t="inlineStr">
+      <c r="H18" s="1" t="inlineStr">
         <is>
           <t>停損</t>
         </is>
@@ -1002,13 +1093,18 @@
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F19" s="1" t="inlineStr">
+        <is>
           <t>等價進場買入</t>
         </is>
       </c>
-      <c r="F19" s="1" t="n">
+      <c r="G19" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G19" s="1" t="inlineStr"/>
+      <c r="H19" s="1" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
@@ -1031,13 +1127,18 @@
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F20" s="1" t="inlineStr">
+        <is>
           <t>23戰法買</t>
         </is>
       </c>
-      <c r="F20" s="1" t="n">
+      <c r="G20" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G20" s="1" t="inlineStr"/>
+      <c r="H20" s="1" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
@@ -1060,13 +1161,18 @@
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F21" s="1" t="inlineStr">
+        <is>
           <t>停損賣出</t>
         </is>
       </c>
-      <c r="F21" s="1" t="n">
+      <c r="G21" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G21" s="1" t="inlineStr">
+      <c r="H21" s="1" t="inlineStr">
         <is>
           <t>停損</t>
         </is>
@@ -1093,13 +1199,18 @@
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F22" s="1" t="inlineStr">
+        <is>
           <t>KD高腳</t>
         </is>
       </c>
-      <c r="F22" s="1" t="n">
+      <c r="G22" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G22" s="1" t="inlineStr"/>
+      <c r="H22" s="1" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
@@ -1122,13 +1233,18 @@
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F23" s="1" t="inlineStr">
+        <is>
           <t>KD高腳</t>
         </is>
       </c>
-      <c r="F23" s="1" t="n">
+      <c r="G23" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G23" s="1" t="inlineStr">
+      <c r="H23" s="1" t="inlineStr">
         <is>
           <t>迴旋KD</t>
         </is>
@@ -1155,13 +1271,18 @@
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F24" s="1" t="inlineStr">
+        <is>
           <t>3K反轉</t>
         </is>
       </c>
-      <c r="F24" s="1" t="n">
+      <c r="G24" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G24" s="1" t="inlineStr"/>
+      <c r="H24" s="1" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
@@ -1184,13 +1305,18 @@
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F25" s="1" t="inlineStr">
+        <is>
           <t>停利賣出</t>
         </is>
       </c>
-      <c r="F25" s="1" t="n">
+      <c r="G25" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="G25" s="1" t="inlineStr"/>
+      <c r="H25" s="1" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
@@ -1213,13 +1339,18 @@
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F26" s="1" t="inlineStr">
+        <is>
           <t>陰K加碼</t>
         </is>
       </c>
-      <c r="F26" s="1" t="n">
+      <c r="G26" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G26" s="1" t="inlineStr"/>
+      <c r="H26" s="1" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
@@ -1242,13 +1373,52 @@
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F27" s="1" t="inlineStr">
+        <is>
           <t>巧妙點</t>
         </is>
       </c>
-      <c r="F27" s="1" t="n">
+      <c r="G27" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G27" s="1" t="inlineStr"/>
+      <c r="H27" s="1" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
+        <is>
+          <t>3362</t>
+        </is>
+      </c>
+      <c r="C28" s="1" t="inlineStr">
+        <is>
+          <t>先進光</t>
+        </is>
+      </c>
+      <c r="D28" s="1" t="n">
+        <v>202</v>
+      </c>
+      <c r="E28" s="1" t="inlineStr">
+        <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F28" s="1" t="inlineStr">
+        <is>
+          <t>停利賣出</t>
+        </is>
+      </c>
+      <c r="G28" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-28 23:35:34
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1419,6 +1419,70 @@
         <v>1</v>
       </c>
       <c r="H28" s="1" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
+        <is>
+          <t>2377</t>
+        </is>
+      </c>
+      <c r="C29" s="1" t="inlineStr">
+        <is>
+          <t>微星</t>
+        </is>
+      </c>
+      <c r="D29" s="1" t="n">
+        <v>155.6</v>
+      </c>
+      <c r="E29" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F29" s="1" t="inlineStr">
+        <is>
+          <t>KD高腳</t>
+        </is>
+      </c>
+      <c r="G29" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="H29" s="1" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr"/>
+      <c r="B30" s="1" t="inlineStr">
+        <is>
+          <t>2377</t>
+        </is>
+      </c>
+      <c r="C30" s="1" t="inlineStr">
+        <is>
+          <t>微星</t>
+        </is>
+      </c>
+      <c r="D30" s="1" t="n">
+        <v>144</v>
+      </c>
+      <c r="E30" s="1" t="inlineStr">
+        <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F30" s="1" t="inlineStr">
+        <is>
+          <t>停損賣出</t>
+        </is>
+      </c>
+      <c r="G30" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="H30" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-28 23:42:30
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -1455,7 +1455,11 @@
       <c r="H29" s="1" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="inlineStr"/>
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
           <t>2377</t>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-01 12:35:58
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1487,6 +1487,40 @@
         <v>3</v>
       </c>
       <c r="H30" s="1" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
+        <is>
+          <t>3605</t>
+        </is>
+      </c>
+      <c r="C31" s="1" t="inlineStr">
+        <is>
+          <t>宏致</t>
+        </is>
+      </c>
+      <c r="D31" s="1" t="n">
+        <v>125.5</v>
+      </c>
+      <c r="E31" s="1" t="inlineStr">
+        <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F31" s="1" t="inlineStr">
+        <is>
+          <t>跌停</t>
+        </is>
+      </c>
+      <c r="G31" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-01 12:38:01
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1521,6 +1521,40 @@
         <v>1</v>
       </c>
       <c r="H31" s="1" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="inlineStr">
+        <is>
+          <t>5351</t>
+        </is>
+      </c>
+      <c r="C32" s="1" t="inlineStr">
+        <is>
+          <t>鈺創</t>
+        </is>
+      </c>
+      <c r="D32" s="1" t="n">
+        <v>121</v>
+      </c>
+      <c r="E32" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F32" s="1" t="inlineStr">
+        <is>
+          <t>KD高腳</t>
+        </is>
+      </c>
+      <c r="G32" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H32" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-02 12:30:59
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1555,6 +1555,40 @@
         <v>1</v>
       </c>
       <c r="H32" s="1" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B33" s="1" t="inlineStr">
+        <is>
+          <t>8039</t>
+        </is>
+      </c>
+      <c r="C33" s="1" t="inlineStr">
+        <is>
+          <t>台虹</t>
+        </is>
+      </c>
+      <c r="D33" s="1" t="n">
+        <v>316.5</v>
+      </c>
+      <c r="E33" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F33" s="1" t="inlineStr">
+        <is>
+          <t>巧妙點</t>
+        </is>
+      </c>
+      <c r="G33" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H33" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-02 12:31:52
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1589,6 +1589,40 @@
         <v>1</v>
       </c>
       <c r="H33" s="1" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B34" s="1" t="inlineStr">
+        <is>
+          <t>2351</t>
+        </is>
+      </c>
+      <c r="C34" s="1" t="inlineStr">
+        <is>
+          <t>順德</t>
+        </is>
+      </c>
+      <c r="D34" s="1" t="n">
+        <v>226</v>
+      </c>
+      <c r="E34" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F34" s="1" t="inlineStr">
+        <is>
+          <t>巧妙點</t>
+        </is>
+      </c>
+      <c r="G34" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-03 10:32:46
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -427,7 +427,7 @@
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
@@ -1623,6 +1623,74 @@
         <v>1</v>
       </c>
       <c r="H34" s="1" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B35" s="1" t="inlineStr">
+        <is>
+          <t>1303</t>
+        </is>
+      </c>
+      <c r="C35" s="1" t="inlineStr">
+        <is>
+          <t>南亞</t>
+        </is>
+      </c>
+      <c r="D35" s="1" t="n">
+        <v>224</v>
+      </c>
+      <c r="E35" s="1" t="inlineStr">
+        <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F35" s="1" t="inlineStr">
+        <is>
+          <t>上升趨勢線跌破</t>
+        </is>
+      </c>
+      <c r="G35" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H35" s="1" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B36" s="1" t="inlineStr">
+        <is>
+          <t>3605</t>
+        </is>
+      </c>
+      <c r="C36" s="1" t="inlineStr">
+        <is>
+          <t>宏致</t>
+        </is>
+      </c>
+      <c r="D36" s="1" t="n">
+        <v>122</v>
+      </c>
+      <c r="E36" s="1" t="inlineStr">
+        <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F36" s="1" t="inlineStr">
+        <is>
+          <t>移動停利</t>
+        </is>
+      </c>
+      <c r="G36" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="H36" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-03 14:04:16
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1691,6 +1691,72 @@
         <v>3</v>
       </c>
       <c r="H36" s="1" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B37" s="1" t="inlineStr">
+        <is>
+          <t>5351</t>
+        </is>
+      </c>
+      <c r="C37" s="1" t="inlineStr">
+        <is>
+          <t>鈺創</t>
+        </is>
+      </c>
+      <c r="D37" s="1" t="n">
+        <v>113</v>
+      </c>
+      <c r="E37" s="1" t="inlineStr">
+        <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F37" s="1" t="inlineStr">
+        <is>
+          <t>停損賣出</t>
+        </is>
+      </c>
+      <c r="G37" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="H37" s="1" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B38" s="1" t="inlineStr">
+        <is>
+          <t>8039</t>
+        </is>
+      </c>
+      <c r="C38" s="1" t="inlineStr">
+        <is>
+          <t>台虹</t>
+        </is>
+      </c>
+      <c r="D38" s="1" t="n">
+        <v>296</v>
+      </c>
+      <c r="E38" s="1" t="inlineStr">
+        <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F38" s="1" t="inlineStr">
+        <is>
+          <t>停損賣出</t>
+        </is>
+      </c>
+      <c r="G38" s="1" t="inlineStr"/>
+      <c r="H38" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-04 15:23:14
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1755,8 +1755,42 @@
           <t>停損賣出</t>
         </is>
       </c>
-      <c r="G38" s="1" t="inlineStr"/>
+      <c r="G38" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="H38" s="1" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B39" s="1" t="inlineStr">
+        <is>
+          <t>1303</t>
+        </is>
+      </c>
+      <c r="C39" s="1" t="inlineStr">
+        <is>
+          <t>南亞</t>
+        </is>
+      </c>
+      <c r="D39" s="1" t="n">
+        <v>219</v>
+      </c>
+      <c r="E39" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F39" s="1" t="inlineStr">
+        <is>
+          <t>等價進場買入</t>
+        </is>
+      </c>
+      <c r="G39" s="1" t="inlineStr"/>
+      <c r="H39" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-04 15:24:13
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -429,7 +429,7 @@
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1786,11 +1786,17 @@
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>等價進場買入</t>
-        </is>
-      </c>
-      <c r="G39" s="1" t="inlineStr"/>
-      <c r="H39" s="1" t="inlineStr"/>
+          <t>巧妙點</t>
+        </is>
+      </c>
+      <c r="G39" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H39" s="1" t="inlineStr">
+        <is>
+          <t>等價219買入</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-04 15:25:44
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -429,7 +429,7 @@
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1795,6 +1795,44 @@
       <c r="H39" s="1" t="inlineStr">
         <is>
           <t>等價219買入</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B40" s="1" t="inlineStr">
+        <is>
+          <t>6147</t>
+        </is>
+      </c>
+      <c r="C40" s="1" t="inlineStr">
+        <is>
+          <t>頎邦</t>
+        </is>
+      </c>
+      <c r="D40" s="1" t="n">
+        <v>187.5</v>
+      </c>
+      <c r="E40" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F40" s="1" t="inlineStr">
+        <is>
+          <t>等價進場買入</t>
+        </is>
+      </c>
+      <c r="G40" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H40" s="1" t="inlineStr">
+        <is>
+          <t>60MA 價格187</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-07 14:18:47
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1835,6 +1835,40 @@
           <t>60MA 價格187</t>
         </is>
       </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B41" s="1" t="inlineStr">
+        <is>
+          <t>3362</t>
+        </is>
+      </c>
+      <c r="C41" s="1" t="inlineStr">
+        <is>
+          <t>先進光</t>
+        </is>
+      </c>
+      <c r="D41" s="1" t="n">
+        <v>190.5</v>
+      </c>
+      <c r="E41" s="1" t="inlineStr">
+        <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F41" s="1" t="inlineStr">
+        <is>
+          <t>停利賣出</t>
+        </is>
+      </c>
+      <c r="G41" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H41" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-07 14:19:20
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1869,6 +1869,40 @@
         <v>1</v>
       </c>
       <c r="H41" s="1" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B42" s="1" t="inlineStr">
+        <is>
+          <t>1303</t>
+        </is>
+      </c>
+      <c r="C42" s="1" t="inlineStr">
+        <is>
+          <t>南亞</t>
+        </is>
+      </c>
+      <c r="D42" s="1" t="n">
+        <v>231</v>
+      </c>
+      <c r="E42" s="1" t="inlineStr">
+        <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F42" s="1" t="inlineStr">
+        <is>
+          <t>停利賣出</t>
+        </is>
+      </c>
+      <c r="G42" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H42" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-07 14:20:19
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1903,6 +1903,38 @@
         <v>1</v>
       </c>
       <c r="H42" s="1" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B43" s="1" t="inlineStr">
+        <is>
+          <t>3605</t>
+        </is>
+      </c>
+      <c r="C43" s="1" t="inlineStr">
+        <is>
+          <t>宏致</t>
+        </is>
+      </c>
+      <c r="D43" s="1" t="n">
+        <v>121</v>
+      </c>
+      <c r="E43" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F43" s="1" t="inlineStr">
+        <is>
+          <t>巧妙點</t>
+        </is>
+      </c>
+      <c r="G43" s="1" t="inlineStr"/>
+      <c r="H43" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-07 14:20:58
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1933,8 +1933,44 @@
           <t>巧妙點</t>
         </is>
       </c>
-      <c r="G43" s="1" t="inlineStr"/>
+      <c r="G43" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="H43" s="1" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B44" s="1" t="inlineStr">
+        <is>
+          <t>6271</t>
+        </is>
+      </c>
+      <c r="C44" s="1" t="inlineStr">
+        <is>
+          <t>同欣電</t>
+        </is>
+      </c>
+      <c r="D44" s="1" t="n">
+        <v>237</v>
+      </c>
+      <c r="E44" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F44" s="1" t="inlineStr">
+        <is>
+          <t>KD高腳</t>
+        </is>
+      </c>
+      <c r="G44" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H44" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-08 14:21:39
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1971,6 +1971,40 @@
         <v>1</v>
       </c>
       <c r="H44" s="1" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B45" s="1" t="inlineStr">
+        <is>
+          <t>6226</t>
+        </is>
+      </c>
+      <c r="C45" s="1" t="inlineStr">
+        <is>
+          <t>光鼎</t>
+        </is>
+      </c>
+      <c r="D45" s="1" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="E45" s="1" t="inlineStr">
+        <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F45" s="1" t="inlineStr">
+        <is>
+          <t>停利賣出</t>
+        </is>
+      </c>
+      <c r="G45" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="H45" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-10 10:37:00
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,17 +419,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -470,6 +471,11 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>零股(股)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Note</t>
         </is>
       </c>
@@ -507,6 +513,7 @@
         <v>1</v>
       </c>
       <c r="H2" s="1" t="inlineStr"/>
+      <c r="I2" s="1" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -541,6 +548,7 @@
         <v>1</v>
       </c>
       <c r="H3" s="1" t="inlineStr"/>
+      <c r="I3" s="1" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -575,6 +583,7 @@
         <v>2</v>
       </c>
       <c r="H4" s="1" t="inlineStr"/>
+      <c r="I4" s="1" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -609,6 +618,7 @@
         <v>1</v>
       </c>
       <c r="H5" s="1" t="inlineStr"/>
+      <c r="I5" s="1" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -642,7 +652,8 @@
       <c r="G6" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H6" s="1" t="inlineStr">
+      <c r="H6" s="1" t="inlineStr"/>
+      <c r="I6" s="1" t="inlineStr">
         <is>
           <t>開盤有巧妙點</t>
         </is>
@@ -681,6 +692,7 @@
         <v>3</v>
       </c>
       <c r="H7" s="1" t="inlineStr"/>
+      <c r="I7" s="1" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -715,6 +727,7 @@
         <v>2</v>
       </c>
       <c r="H8" s="1" t="inlineStr"/>
+      <c r="I8" s="1" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -749,6 +762,7 @@
         <v>3</v>
       </c>
       <c r="H9" s="1" t="inlineStr"/>
+      <c r="I9" s="1" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -783,6 +797,7 @@
         <v>1</v>
       </c>
       <c r="H10" s="1" t="inlineStr"/>
+      <c r="I10" s="1" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -817,6 +832,7 @@
         <v>1</v>
       </c>
       <c r="H11" s="1" t="inlineStr"/>
+      <c r="I11" s="1" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -851,6 +867,7 @@
         <v>10</v>
       </c>
       <c r="H12" s="1" t="inlineStr"/>
+      <c r="I12" s="1" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -884,7 +901,8 @@
       <c r="G13" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H13" s="1" t="inlineStr">
+      <c r="H13" s="1" t="inlineStr"/>
+      <c r="I13" s="1" t="inlineStr">
         <is>
           <t>停損</t>
         </is>
@@ -922,7 +940,8 @@
       <c r="G14" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H14" s="1" t="inlineStr">
+      <c r="H14" s="1" t="inlineStr"/>
+      <c r="I14" s="1" t="inlineStr">
         <is>
           <t>停利</t>
         </is>
@@ -961,6 +980,7 @@
         <v>2</v>
       </c>
       <c r="H15" s="1" t="inlineStr"/>
+      <c r="I15" s="1" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
@@ -995,6 +1015,7 @@
         <v>3</v>
       </c>
       <c r="H16" s="1" t="inlineStr"/>
+      <c r="I16" s="1" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
@@ -1028,7 +1049,8 @@
       <c r="G17" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H17" s="1" t="inlineStr">
+      <c r="H17" s="1" t="inlineStr"/>
+      <c r="I17" s="1" t="inlineStr">
         <is>
           <t>乖離過大調節</t>
         </is>
@@ -1066,7 +1088,8 @@
       <c r="G18" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="H18" s="1" t="inlineStr">
+      <c r="H18" s="1" t="inlineStr"/>
+      <c r="I18" s="1" t="inlineStr">
         <is>
           <t>停損</t>
         </is>
@@ -1105,6 +1128,7 @@
         <v>1</v>
       </c>
       <c r="H19" s="1" t="inlineStr"/>
+      <c r="I19" s="1" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
@@ -1139,6 +1163,7 @@
         <v>1</v>
       </c>
       <c r="H20" s="1" t="inlineStr"/>
+      <c r="I20" s="1" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
@@ -1172,7 +1197,8 @@
       <c r="G21" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="H21" s="1" t="inlineStr">
+      <c r="H21" s="1" t="inlineStr"/>
+      <c r="I21" s="1" t="inlineStr">
         <is>
           <t>停損</t>
         </is>
@@ -1211,6 +1237,7 @@
         <v>1</v>
       </c>
       <c r="H22" s="1" t="inlineStr"/>
+      <c r="I22" s="1" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
@@ -1244,7 +1271,8 @@
       <c r="G23" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H23" s="1" t="inlineStr">
+      <c r="H23" s="1" t="inlineStr"/>
+      <c r="I23" s="1" t="inlineStr">
         <is>
           <t>迴旋KD</t>
         </is>
@@ -1283,6 +1311,7 @@
         <v>1</v>
       </c>
       <c r="H24" s="1" t="inlineStr"/>
+      <c r="I24" s="1" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
@@ -1317,6 +1346,7 @@
         <v>3</v>
       </c>
       <c r="H25" s="1" t="inlineStr"/>
+      <c r="I25" s="1" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
@@ -1351,6 +1381,7 @@
         <v>1</v>
       </c>
       <c r="H26" s="1" t="inlineStr"/>
+      <c r="I26" s="1" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
@@ -1385,6 +1416,7 @@
         <v>1</v>
       </c>
       <c r="H27" s="1" t="inlineStr"/>
+      <c r="I27" s="1" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
@@ -1419,6 +1451,7 @@
         <v>1</v>
       </c>
       <c r="H28" s="1" t="inlineStr"/>
+      <c r="I28" s="1" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
@@ -1453,6 +1486,7 @@
         <v>3</v>
       </c>
       <c r="H29" s="1" t="inlineStr"/>
+      <c r="I29" s="1" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
@@ -1487,6 +1521,7 @@
         <v>3</v>
       </c>
       <c r="H30" s="1" t="inlineStr"/>
+      <c r="I30" s="1" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
@@ -1521,6 +1556,7 @@
         <v>1</v>
       </c>
       <c r="H31" s="1" t="inlineStr"/>
+      <c r="I31" s="1" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
@@ -1555,6 +1591,7 @@
         <v>1</v>
       </c>
       <c r="H32" s="1" t="inlineStr"/>
+      <c r="I32" s="1" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
@@ -1589,6 +1626,7 @@
         <v>1</v>
       </c>
       <c r="H33" s="1" t="inlineStr"/>
+      <c r="I33" s="1" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
@@ -1623,6 +1661,7 @@
         <v>1</v>
       </c>
       <c r="H34" s="1" t="inlineStr"/>
+      <c r="I34" s="1" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
@@ -1657,6 +1696,7 @@
         <v>1</v>
       </c>
       <c r="H35" s="1" t="inlineStr"/>
+      <c r="I35" s="1" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
@@ -1691,6 +1731,7 @@
         <v>3</v>
       </c>
       <c r="H36" s="1" t="inlineStr"/>
+      <c r="I36" s="1" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
@@ -1725,6 +1766,7 @@
         <v>2</v>
       </c>
       <c r="H37" s="1" t="inlineStr"/>
+      <c r="I37" s="1" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
@@ -1759,6 +1801,7 @@
         <v>1</v>
       </c>
       <c r="H38" s="1" t="inlineStr"/>
+      <c r="I38" s="1" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
@@ -1792,7 +1835,8 @@
       <c r="G39" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H39" s="1" t="inlineStr">
+      <c r="H39" s="1" t="inlineStr"/>
+      <c r="I39" s="1" t="inlineStr">
         <is>
           <t>等價219買入</t>
         </is>
@@ -1830,7 +1874,8 @@
       <c r="G40" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H40" s="1" t="inlineStr">
+      <c r="H40" s="1" t="inlineStr"/>
+      <c r="I40" s="1" t="inlineStr">
         <is>
           <t>60MA 價格187</t>
         </is>
@@ -1869,6 +1914,7 @@
         <v>1</v>
       </c>
       <c r="H41" s="1" t="inlineStr"/>
+      <c r="I41" s="1" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
@@ -1903,6 +1949,7 @@
         <v>1</v>
       </c>
       <c r="H42" s="1" t="inlineStr"/>
+      <c r="I42" s="1" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
@@ -1937,6 +1984,7 @@
         <v>1</v>
       </c>
       <c r="H43" s="1" t="inlineStr"/>
+      <c r="I43" s="1" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
@@ -1971,6 +2019,7 @@
         <v>1</v>
       </c>
       <c r="H44" s="1" t="inlineStr"/>
+      <c r="I44" s="1" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
@@ -2005,6 +2054,42 @@
         <v>10</v>
       </c>
       <c r="H45" s="1" t="inlineStr"/>
+      <c r="I45" s="1" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B46" s="1" t="inlineStr">
+        <is>
+          <t>3081</t>
+        </is>
+      </c>
+      <c r="C46" s="1" t="inlineStr">
+        <is>
+          <t>聯亞</t>
+        </is>
+      </c>
+      <c r="D46" s="1" t="n">
+        <v>2875.5</v>
+      </c>
+      <c r="E46" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F46" s="1" t="inlineStr">
+        <is>
+          <t>巧妙點</t>
+        </is>
+      </c>
+      <c r="G46" s="1" t="inlineStr"/>
+      <c r="H46" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="I46" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-10 10:41:45
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2090,6 +2090,41 @@
         <v>90</v>
       </c>
       <c r="I46" s="1" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B47" s="1" t="inlineStr">
+        <is>
+          <t>3605</t>
+        </is>
+      </c>
+      <c r="C47" s="1" t="inlineStr">
+        <is>
+          <t>宏致</t>
+        </is>
+      </c>
+      <c r="D47" s="1" t="n">
+        <v>130</v>
+      </c>
+      <c r="E47" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F47" s="1" t="inlineStr">
+        <is>
+          <t>KD高腳</t>
+        </is>
+      </c>
+      <c r="G47" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H47" s="1" t="inlineStr"/>
+      <c r="I47" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-11 09:48:25
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2125,6 +2125,41 @@
       </c>
       <c r="H47" s="1" t="inlineStr"/>
       <c r="I47" s="1" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B48" s="1" t="inlineStr">
+        <is>
+          <t>8261</t>
+        </is>
+      </c>
+      <c r="C48" s="1" t="inlineStr">
+        <is>
+          <t>富鼎</t>
+        </is>
+      </c>
+      <c r="D48" s="1" t="n">
+        <v>162.5</v>
+      </c>
+      <c r="E48" s="1" t="inlineStr">
+        <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F48" s="1" t="inlineStr">
+        <is>
+          <t>停損賣出</t>
+        </is>
+      </c>
+      <c r="G48" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H48" s="1" t="inlineStr"/>
+      <c r="I48" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-11 11:10:11
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2160,6 +2160,41 @@
       </c>
       <c r="H48" s="1" t="inlineStr"/>
       <c r="I48" s="1" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B49" s="1" t="inlineStr">
+        <is>
+          <t>2351</t>
+        </is>
+      </c>
+      <c r="C49" s="1" t="inlineStr">
+        <is>
+          <t>順德</t>
+        </is>
+      </c>
+      <c r="D49" s="1" t="n">
+        <v>232.5</v>
+      </c>
+      <c r="E49" s="1" t="inlineStr">
+        <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F49" s="1" t="inlineStr">
+        <is>
+          <t>停利賣出</t>
+        </is>
+      </c>
+      <c r="G49" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H49" s="1" t="inlineStr"/>
+      <c r="I49" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>